<commit_message>
capitalise, progressive number inserted
</commit_message>
<xml_diff>
--- a/production_BOM/bom_r3_cust.xlsx
+++ b/production_BOM/bom_r3_cust.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git-repos\cad-libraries\production_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318F6180-D5C6-4B29-83D1-21084776CB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEC49449-0BBA-460A-905B-DAB5999DFAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24000" yWindow="0" windowWidth="24195" windowHeight="14280" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="components request" sheetId="1" r:id="rId1"/>
@@ -102,10 +102,10 @@
     <t>Other</t>
   </si>
   <si>
-    <t>test_rev_0</t>
-  </si>
-  <si>
-    <t>test_rev_A2</t>
+    <t>EXAMPLE1_REV_0</t>
+  </si>
+  <si>
+    <t>EXAMPLE2_REV_A2</t>
   </si>
 </sst>
 </file>
@@ -618,6 +618,9 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2" t="s">
         <v>21</v>
       </c>
@@ -627,6 +630,9 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
       <c r="B3" t="s">
         <v>22</v>
       </c>

</xml_diff>